<commit_message>
Plotting Task 3 graphs
</commit_message>
<xml_diff>
--- a/graph/RunningTimeRecord.xlsx
+++ b/graph/RunningTimeRecord.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chtay\Documents\FIT3143\FIT3143_lab01\graph\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C4B56E-1352-40AA-98A0-2B0DE9B68D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15BA1BAF-E601-47E0-808D-ACCAB26369FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Testing 1" sheetId="1" r:id="rId1"/>
@@ -1960,14 +1960,15 @@
         <v>1</v>
       </c>
       <c r="B5" s="6">
-        <v>4.221819</v>
+        <f>'Testing 1'!$B$5</f>
+        <v>1.981976</v>
       </c>
       <c r="C5">
         <v>1.9988060000000001</v>
       </c>
       <c r="D5" s="6">
         <f>B5/C5</f>
-        <v>2.1121704657680636</v>
+        <v>0.99157997324402658</v>
       </c>
       <c r="E5">
         <v>2.0506150000000001</v>
@@ -1978,14 +1979,15 @@
         <v>4</v>
       </c>
       <c r="B6" s="6">
-        <v>4.221819</v>
+        <f>'Testing 1'!$B$5</f>
+        <v>1.981976</v>
       </c>
       <c r="C6">
         <v>1.163114</v>
       </c>
       <c r="D6" s="6">
         <f t="shared" ref="D6:D10" si="0">B6/C6</f>
-        <v>3.6297551228856331</v>
+        <v>1.7040255727297582</v>
       </c>
       <c r="E6">
         <v>0.62085500000000005</v>
@@ -1996,14 +1998,15 @@
         <v>8</v>
       </c>
       <c r="B7" s="6">
-        <v>4.221819</v>
+        <f>'Testing 1'!$B$5</f>
+        <v>1.981976</v>
       </c>
       <c r="C7">
         <v>0.66360600000000003</v>
       </c>
       <c r="D7" s="6">
         <f t="shared" si="0"/>
-        <v>6.3619361488594128</v>
+        <v>2.9866758287296977</v>
       </c>
       <c r="E7">
         <v>0.39751399999999998</v>
@@ -2014,14 +2017,15 @@
         <v>16</v>
       </c>
       <c r="B8" s="6">
-        <v>4.221819</v>
+        <f>'Testing 1'!$B$5</f>
+        <v>1.981976</v>
       </c>
       <c r="C8">
         <v>0.445718</v>
       </c>
       <c r="D8" s="6">
         <f t="shared" si="0"/>
-        <v>9.4719508747683516</v>
+        <v>4.4467039697746111</v>
       </c>
       <c r="E8">
         <v>0.39396199999999998</v>
@@ -2032,14 +2036,15 @@
         <v>32</v>
       </c>
       <c r="B9" s="6">
-        <v>4.221819</v>
+        <f>'Testing 1'!$B$5</f>
+        <v>1.981976</v>
       </c>
       <c r="C9">
         <v>0.44677899999999998</v>
       </c>
       <c r="D9" s="6">
         <f t="shared" si="0"/>
-        <v>9.4494571141436818</v>
+        <v>4.4361440443709306</v>
       </c>
       <c r="E9">
         <v>0.40589199999999998</v>
@@ -2050,14 +2055,15 @@
         <v>64</v>
       </c>
       <c r="B10" s="6">
-        <v>4.221819</v>
+        <f>'Testing 1'!$B$5</f>
+        <v>1.981976</v>
       </c>
       <c r="C10">
         <v>0.44517200000000001</v>
       </c>
       <c r="D10" s="6">
         <f t="shared" si="0"/>
-        <v>9.4835681489401846</v>
+        <v>4.4521578176525027</v>
       </c>
       <c r="E10">
         <v>0.40879700000000002</v>
@@ -2107,14 +2113,15 @@
         <v>1</v>
       </c>
       <c r="B16" s="6">
-        <v>1.819431</v>
+        <f>'Testing 1'!$B$40</f>
+        <v>1.909535</v>
       </c>
       <c r="C16">
         <v>1.7803150000000001</v>
       </c>
       <c r="D16" s="6">
         <f>B16/C16</f>
-        <v>1.0219713927029768</v>
+        <v>1.0725826609335987</v>
       </c>
       <c r="E16">
         <v>1.794886</v>
@@ -2125,14 +2132,15 @@
         <v>4</v>
       </c>
       <c r="B17" s="6">
-        <v>1.819431</v>
+        <f>'Testing 1'!$B$40</f>
+        <v>1.909535</v>
       </c>
       <c r="C17">
         <v>0.91214399999999995</v>
       </c>
       <c r="D17" s="6">
         <f t="shared" ref="D17:D21" si="1">B17/C17</f>
-        <v>1.9946751828658633</v>
+        <v>2.0934578312196321</v>
       </c>
       <c r="E17">
         <v>0.43836999999999998</v>
@@ -2143,14 +2151,15 @@
         <v>8</v>
       </c>
       <c r="B18" s="6">
-        <v>1.819431</v>
+        <f>'Testing 1'!$B$40</f>
+        <v>1.909535</v>
       </c>
       <c r="C18">
         <v>0.41222500000000001</v>
       </c>
       <c r="D18" s="6">
         <f t="shared" si="1"/>
-        <v>4.4136842743647282</v>
+        <v>4.6322639335314451</v>
       </c>
       <c r="E18">
         <v>0.225991</v>
@@ -2161,14 +2170,15 @@
         <v>16</v>
       </c>
       <c r="B19" s="6">
-        <v>1.819431</v>
+        <f>'Testing 1'!$B$40</f>
+        <v>1.909535</v>
       </c>
       <c r="C19">
         <v>0.248222</v>
       </c>
       <c r="D19" s="6">
         <f t="shared" si="1"/>
-        <v>7.3298539210867695</v>
+        <v>7.6928515602968313</v>
       </c>
       <c r="E19">
         <v>0.15532199999999999</v>
@@ -2179,14 +2189,15 @@
         <v>32</v>
       </c>
       <c r="B20" s="6">
-        <v>1.819431</v>
+        <f>'Testing 1'!$B$40</f>
+        <v>1.909535</v>
       </c>
       <c r="C20">
         <v>0.18618000000000001</v>
       </c>
       <c r="D20" s="6">
         <f t="shared" si="1"/>
-        <v>9.7724299065420563</v>
+        <v>10.256391663981093</v>
       </c>
       <c r="E20">
         <v>0.14178299999999999</v>
@@ -2197,14 +2208,15 @@
         <v>64</v>
       </c>
       <c r="B21" s="6">
-        <v>1.819431</v>
+        <f>'Testing 1'!$B$40</f>
+        <v>1.909535</v>
       </c>
       <c r="C21">
         <v>0.175349</v>
       </c>
       <c r="D21" s="6">
         <f t="shared" si="1"/>
-        <v>10.376055751672379</v>
+        <v>10.889910977536227</v>
       </c>
       <c r="E21">
         <v>0.141709</v>

</xml_diff>